<commit_message>
found some points to improve. Works better now.
</commit_message>
<xml_diff>
--- a/SolutionFiles/results.xlsx
+++ b/SolutionFiles/results.xlsx
@@ -486,14 +486,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>rc207_21.txt</t>
+          <t>r202C15.txt</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>149.6000508443449</v>
+        <v>79.27096704353858</v>
       </c>
       <c r="D2" t="n">
-        <v>1063.46684804547</v>
+        <v>621.8301118421625</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -504,19 +504,19 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>25000</v>
+        <v>10</v>
       </c>
       <c r="H2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I2" t="n">
         <v>5</v>
-      </c>
-      <c r="I2" t="n">
-        <v>4</v>
       </c>
       <c r="J2" t="n">
         <v>50</v>
       </c>
       <c r="K2" t="n">
-        <v>106403.8963594437</v>
+        <v>3.267267465591431</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
esogu dataset read and some more improvements
</commit_message>
<xml_diff>
--- a/SolutionFiles/results.xlsx
+++ b/SolutionFiles/results.xlsx
@@ -486,14 +486,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>c105_21.txt</t>
+          <t>ESOGU_C10_TW1.txt</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>196.9190957526799</v>
+        <v>21602.9098491384</v>
       </c>
       <c r="D2" t="n">
-        <v>1500.116272611965</v>
+        <v>87217.04720116501</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -504,7 +504,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>25000</v>
       </c>
       <c r="H2" t="n">
         <v>20</v>
@@ -513,10 +513,10 @@
         <v>10</v>
       </c>
       <c r="J2" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="K2" t="n">
-        <v>155.7044532299042</v>
+        <v>198.704959154129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>